<commit_message>
feat(build): rework Makefile and add multi-target VSCode tasks
</commit_message>
<xml_diff>
--- a/benchmarks.xlsx
+++ b/benchmarks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OpenSource\z88dk-bench\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369488B3-C0EE-406A-8666-8926DCCEB67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A63C50-ED75-416C-9348-5FADA19AE343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="21">
   <si>
     <t>compiler</t>
   </si>
@@ -98,6 +98,12 @@
   <si>
     <t>Suma de  time(ms)</t>
   </si>
+  <si>
+    <t>sccz80-classic</t>
+  </si>
+  <si>
+    <t>sccz80-new</t>
+  </si>
 </sst>
 </file>
 
@@ -120,7 +126,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -128,31 +134,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <alignment horizontal="right"/>
     </dxf>
@@ -192,7 +204,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[graph.xlsx]Graph!TablaDinámica2</c:name>
+    <c:name>[benchmarks.xlsx]Graph!TablaDinámica2</c:name>
     <c:fmtId val="1"/>
   </c:pivotSource>
   <c:chart>
@@ -1560,7 +1572,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2AFB877-D027-4C90-A4D4-A68E510C4F5E}" name="TablaDinámica2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2AFB877-D027-4C90-A4D4-A68E510C4F5E}" name="TablaDinámica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField axis="axisCol" showAll="0">
@@ -1624,7 +1636,7 @@
     <dataField name="Suma de  time(ms)" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="1">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -1719,16 +1731,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CCBFCE38-E217-4E83-91A4-4A43DD150E92}" name="results" displayName="results" ref="A1:G13" totalsRowShown="0">
-  <autoFilter ref="A1:G13" xr:uid="{CCBFCE38-E217-4E83-91A4-4A43DD150E92}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CCBFCE38-E217-4E83-91A4-4A43DD150E92}" name="results" displayName="results" ref="A1:G9" totalsRowShown="0">
+  <autoFilter ref="A1:G9" xr:uid="{CCBFCE38-E217-4E83-91A4-4A43DD150E92}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{3D679AED-620D-4110-A991-6FE5D6DE6A38}" name="compiler" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{3D679AED-620D-4110-A991-6FE5D6DE6A38}" name="compiler" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{50CD3935-8BD4-43D7-8C4F-E8010D4496F7}" name=" compiled-size"/>
     <tableColumn id="3" xr3:uid="{65493495-318F-4397-B5F1-1CC27DA75D1A}" name=" tap-size"/>
     <tableColumn id="4" xr3:uid="{3E10629F-C516-4743-A105-3A8D754E487B}" name=" empty-project-tap-size"/>
-    <tableColumn id="5" xr3:uid="{B7B7CF54-810C-43DF-9C0D-297A0887CEC4}" name=" test" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{B7B7CF54-810C-43DF-9C0D-297A0887CEC4}" name=" test" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{EE01FD54-F3D2-4FA9-A6C3-225B2EEE4C47}" name=" time(ms)"/>
-    <tableColumn id="7" xr3:uid="{1E91D168-52EA-41CF-9995-EA8F45942C63}" name="Column1" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{1E91D168-52EA-41CF-9995-EA8F45942C63}" name="Column1" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1997,10 +2009,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ECF1D74-EDE2-4E13-B07C-5B1FAA680F97}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -2218,22 +2230,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10">
-        <v>2523</v>
-      </c>
-      <c r="C10">
-        <v>4996</v>
-      </c>
-      <c r="D10">
-        <v>2131</v>
+        <v>20</v>
+      </c>
+      <c r="D10" s="4">
+        <v>554</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
-      </c>
-      <c r="F10">
-        <v>5640</v>
       </c>
       <c r="G10" t="s">
         <v>9</v>
@@ -2241,22 +2244,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11">
-        <v>2523</v>
-      </c>
-      <c r="C11">
-        <v>4996</v>
-      </c>
-      <c r="D11">
-        <v>2131</v>
+        <v>20</v>
+      </c>
+      <c r="D11" s="4">
+        <v>554</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
-      </c>
-      <c r="F11">
-        <v>3500</v>
       </c>
       <c r="G11" t="s">
         <v>9</v>
@@ -2264,22 +2258,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>2523</v>
-      </c>
-      <c r="C12">
-        <v>4996</v>
-      </c>
-      <c r="D12">
-        <v>2131</v>
+        <v>20</v>
+      </c>
+      <c r="D12" s="4">
+        <v>554</v>
       </c>
       <c r="E12" t="s">
         <v>11</v>
-      </c>
-      <c r="F12">
-        <v>3480</v>
       </c>
       <c r="G12" t="s">
         <v>9</v>
@@ -2287,31 +2272,116 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13">
-        <v>2523</v>
-      </c>
-      <c r="C13">
-        <v>4996</v>
-      </c>
-      <c r="D13">
-        <v>2131</v>
+        <v>20</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="D13" s="4">
+        <v>554</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
       </c>
-      <c r="F13">
+      <c r="G13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
+        <v>2523</v>
+      </c>
+      <c r="C14">
+        <v>4996</v>
+      </c>
+      <c r="D14">
+        <v>2131</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14">
+        <v>5640</v>
+      </c>
+      <c r="G14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15">
+        <v>2523</v>
+      </c>
+      <c r="C15">
+        <v>4996</v>
+      </c>
+      <c r="D15">
+        <v>2131</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15">
+        <v>3500</v>
+      </c>
+      <c r="G15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16">
+        <v>2523</v>
+      </c>
+      <c r="C16">
+        <v>4996</v>
+      </c>
+      <c r="D16">
+        <v>2131</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16">
+        <v>3480</v>
+      </c>
+      <c r="G16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>2523</v>
+      </c>
+      <c r="C17">
+        <v>4996</v>
+      </c>
+      <c r="D17">
+        <v>2131</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17">
         <v>4060</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G17" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2346,13 +2416,13 @@
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2360,13 +2430,13 @@
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>5640</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>3120</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
         <v>3060</v>
       </c>
     </row>
@@ -2374,13 +2444,13 @@
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6">
         <v>4060</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6">
         <v>1540</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6">
         <v>1560</v>
       </c>
     </row>
@@ -2388,13 +2458,13 @@
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>3500</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>3220</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7">
         <v>3180</v>
       </c>
     </row>
@@ -2402,13 +2472,13 @@
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>3480</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8">
         <v>3220</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8">
         <v>3180</v>
       </c>
     </row>
@@ -2416,13 +2486,13 @@
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9">
         <v>16680</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9">
         <v>11100</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9">
         <v>10980</v>
       </c>
     </row>

</xml_diff>